<commit_message>
Add WNBA support to split script; correct NBA/WNBA historical colors per TruColor
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\TRACERsports\DBs\wnba\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3BE862-7B53-4987-916E-EAAE27925868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965A25A3-FB99-4083-9435-3BC0AB26DB4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1654EDFA-4626-4D72-A032-E72CC9A130FE}"/>
   </bookViews>
@@ -16588,6 +16588,15 @@
       <c r="G502" t="s">
         <v>24</v>
       </c>
+      <c r="H502">
+        <v>104</v>
+      </c>
+      <c r="I502">
+        <v>69</v>
+      </c>
+      <c r="J502">
+        <v>0</v>
+      </c>
     </row>
     <row r="503" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A503" s="1">
@@ -16611,6 +16620,15 @@
       <c r="G503" t="s">
         <v>25</v>
       </c>
+      <c r="H503">
+        <v>69</v>
+      </c>
+      <c r="I503">
+        <v>104</v>
+      </c>
+      <c r="J503">
+        <v>0</v>
+      </c>
     </row>
     <row r="504" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A504" s="1">
@@ -16634,6 +16652,15 @@
       <c r="G504" t="s">
         <v>24</v>
       </c>
+      <c r="H504">
+        <v>76</v>
+      </c>
+      <c r="I504">
+        <v>83</v>
+      </c>
+      <c r="J504">
+        <v>0</v>
+      </c>
     </row>
     <row r="505" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A505" s="1">
@@ -16657,6 +16684,15 @@
       <c r="G505" t="s">
         <v>25</v>
       </c>
+      <c r="H505">
+        <v>83</v>
+      </c>
+      <c r="I505">
+        <v>76</v>
+      </c>
+      <c r="J505">
+        <v>0</v>
+      </c>
     </row>
     <row r="506" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A506" s="1">
@@ -16680,6 +16716,15 @@
       <c r="G506" t="s">
         <v>24</v>
       </c>
+      <c r="H506">
+        <v>81</v>
+      </c>
+      <c r="I506">
+        <v>85</v>
+      </c>
+      <c r="J506">
+        <v>0</v>
+      </c>
     </row>
     <row r="507" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A507" s="1">
@@ -16702,6 +16747,15 @@
       </c>
       <c r="G507" t="s">
         <v>25</v>
+      </c>
+      <c r="H507">
+        <v>85</v>
+      </c>
+      <c r="I507">
+        <v>81</v>
+      </c>
+      <c r="J507">
+        <v>0</v>
       </c>
     </row>
     <row r="508" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Mix Up Clean Up
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\TRACERsports\DBs\wnba\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC163805-3337-492D-9619-A2ACF60A1064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99A1AC3-7A60-4FBA-B051-95BC6DF96473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1654EDFA-4626-4D72-A032-E72CC9A130FE}"/>
   </bookViews>
@@ -16973,10 +16973,10 @@
         <v>24</v>
       </c>
       <c r="H514">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="I514">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="J514">
         <v>0</v>
@@ -17005,10 +17005,10 @@
         <v>25</v>
       </c>
       <c r="H515">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="I515">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="J515">
         <v>0</v>
@@ -17037,10 +17037,10 @@
         <v>24</v>
       </c>
       <c r="H516">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="I516">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="J516">
         <v>0</v>
@@ -17069,10 +17069,10 @@
         <v>25</v>
       </c>
       <c r="H517">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="I517">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="J517">
         <v>0</v>

</xml_diff>

<commit_message>
Add 2026-08-29 results and Mobile Layout
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -25342,6 +25342,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H592" t="n">
+        <v>66</v>
+      </c>
+      <c r="I592" t="n">
+        <v>85</v>
+      </c>
+      <c r="J592" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="593">
       <c r="A593" s="1" t="n">
@@ -25375,6 +25384,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H593" t="n">
+        <v>85</v>
+      </c>
+      <c r="I593" t="n">
+        <v>66</v>
+      </c>
+      <c r="J593" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="594">
       <c r="A594" s="1" t="n">
@@ -25408,6 +25426,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H594" t="n">
+        <v>69</v>
+      </c>
+      <c r="I594" t="n">
+        <v>101</v>
+      </c>
+      <c r="J594" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="595">
       <c r="A595" s="1" t="n">
@@ -25440,6 +25467,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H595" t="n">
+        <v>101</v>
+      </c>
+      <c r="I595" t="n">
+        <v>69</v>
+      </c>
+      <c r="J595" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="596">

</xml_diff>

<commit_message>
Add 2026-08-30 results and Season Preview
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2026_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2026_Results.xlsx
@@ -25510,6 +25510,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H596" t="n">
+        <v>81</v>
+      </c>
+      <c r="I596" t="n">
+        <v>89</v>
+      </c>
+      <c r="J596" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="597">
       <c r="A597" s="1" t="n">
@@ -25543,6 +25552,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H597" t="n">
+        <v>89</v>
+      </c>
+      <c r="I597" t="n">
+        <v>81</v>
+      </c>
+      <c r="J597" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="598">
       <c r="A598" s="1" t="n">
@@ -25576,6 +25594,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H598" t="n">
+        <v>71</v>
+      </c>
+      <c r="I598" t="n">
+        <v>97</v>
+      </c>
+      <c r="J598" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="599">
       <c r="A599" s="1" t="n">
@@ -25609,6 +25636,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H599" t="n">
+        <v>97</v>
+      </c>
+      <c r="I599" t="n">
+        <v>71</v>
+      </c>
+      <c r="J599" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="600">
       <c r="A600" s="1" t="n">
@@ -25642,6 +25678,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H600" t="n">
+        <v>86</v>
+      </c>
+      <c r="I600" t="n">
+        <v>69</v>
+      </c>
+      <c r="J600" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="601">
       <c r="A601" s="1" t="n">
@@ -25675,6 +25720,15 @@
           <t>H</t>
         </is>
       </c>
+      <c r="H601" t="n">
+        <v>69</v>
+      </c>
+      <c r="I601" t="n">
+        <v>86</v>
+      </c>
+      <c r="J601" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="602">
       <c r="A602" s="1" t="n">
@@ -25708,6 +25762,15 @@
           <t>A</t>
         </is>
       </c>
+      <c r="H602" t="n">
+        <v>90</v>
+      </c>
+      <c r="I602" t="n">
+        <v>74</v>
+      </c>
+      <c r="J602" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="603">
       <c r="A603" s="1" t="n">
@@ -25740,6 +25803,15 @@
         <is>
           <t>H</t>
         </is>
+      </c>
+      <c r="H603" t="n">
+        <v>74</v>
+      </c>
+      <c r="I603" t="n">
+        <v>90</v>
+      </c>
+      <c r="J603" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="604">

</xml_diff>